<commit_message>
Docs: the module dashboards, and companies on the user edit form
Acceptance scripts, 87 → 94 checks: ADM-11 (give someone a second company,
and at least one must stay ticked), ADM-12 (one company is still shown),
EST-13, SITE-05, STR-12, FC-07 and HR-10 (each dashboard agrees with the
screens behind it, shows only that role's figures, and the HR one no
salary). TK-02 expects the HR & Admin entry opening a muster-only dashboard.

Handbook: a section on the module dashboards, the one-company filter, and
changing someone's companies; Finance → Accounts, the renamed tab. In-app
help: a "Module dashboards" article on each dashboard. Workbook and
Handbook PDF rebuilt (94 checks, verified; 46 pages).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/White_and_Bright_ERP_Acceptance_Scripts.xlsx
+++ b/docs/White_and_Bright_ERP_Acceptance_Scripts.xlsx
@@ -23,27 +23,27 @@
     <sheet name="Site Timekeeper" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Administrator'!$A$7:$K$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Administrator'!$A$7:$K$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Administrator'!$7:$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Estimator - Sales'!$A$7:$K$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Estimator - Sales'!$A$7:$K$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Estimator - Sales'!$7:$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Operations &amp; Directors'!$A$7:$K$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Operations &amp; Directors'!$7:$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Site Engineer'!$A$7:$K$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Site Engineer'!$A$7:$K$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Site Engineer'!$7:$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Project Manager'!$A$7:$K$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Project Manager'!$7:$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Procurement'!$A$7:$K$17</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Procurement'!$7:$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Storekeeper'!$A$7:$K$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Storekeeper'!$A$7:$K$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'Storekeeper'!$7:$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'QA-QC &amp; Calibration'!$A$7:$K$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">'QA-QC &amp; Calibration'!$7:$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Accounts'!$A$7:$K$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="10">'Accounts'!$7:$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Finance Controller'!$A$7:$K$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Finance Controller'!$A$7:$K$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="11">'Finance Controller'!$7:$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'HR'!$A$7:$K$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'HR'!$A$7:$K$17</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="12">'HR'!$7:$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Site Timekeeper'!$A$7:$K$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="13">'Site Timekeeper'!$7:$7</definedName>
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>User acceptance testing in Pre-Prod · September 2026 · 87 checks across 12 roles</t>
+          <t>User acceptance testing in Pre-Prod · September 2026 · 94 checks across 12 roles</t>
         </is>
       </c>
     </row>
@@ -1950,7 +1950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2236,10 +2236,10 @@
       <c r="J12" s="41" t="n"/>
       <c r="K12" s="42" t="n"/>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13" ht="87" customHeight="1">
       <c r="A13" s="37" t="inlineStr">
         <is>
-          <t>FC-06</t>
+          <t>FC-07</t>
         </is>
       </c>
       <c r="B13" s="38" t="inlineStr">
@@ -2249,38 +2249,73 @@
       </c>
       <c r="C13" s="39" t="inlineStr">
         <is>
-          <t>Approve the payroll run HR prepared</t>
+          <t>The finance dashboard agrees with the reports</t>
         </is>
       </c>
       <c r="D13" s="38" t="inlineStr">
         <is>
-          <t>1. Open HR → Payroll. Find the run HR prepared in HR-03 and check the totals.
-2. Click Approve. Then Mark paid.</t>
+          <t>1. Click Finance &amp; Accounting in the menu. It opens on the Dashboard tab.
+2. Note Income this year, Profit this year and Customers owe us.
+3. Open Reports → Profit &amp; Loss for 1 January to today, then Outstanding &amp; Ageing.</t>
         </is>
       </c>
       <c r="E13" s="38" t="inlineStr">
         <is>
-          <t>The run is Approved, then Paid, and the wage cost is posted to the books. HR can prepare a run but not approve it, so the salary run is always checked by a second person.</t>
-        </is>
-      </c>
-      <c r="F13" s="40" t="inlineStr">
-        <is>
-          <t>Needs HR-03.</t>
-        </is>
-      </c>
+          <t>Income and profit on the dashboard equal the Profit &amp; Loss for the year to date. Customers owe us equals the receivables total on Outstanding &amp; Ageing. Each tile opens the screen its figure comes from.</t>
+        </is>
+      </c>
+      <c r="F13" s="40" t="inlineStr"/>
       <c r="G13" s="41" t="n"/>
       <c r="H13" s="41" t="n"/>
       <c r="I13" s="41" t="n"/>
       <c r="J13" s="41" t="n"/>
       <c r="K13" s="42" t="n"/>
     </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="37" t="inlineStr">
+        <is>
+          <t>FC-06</t>
+        </is>
+      </c>
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>Finance &amp; HR</t>
+        </is>
+      </c>
+      <c r="C14" s="39" t="inlineStr">
+        <is>
+          <t>Approve the payroll run HR prepared</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
+        <is>
+          <t>1. Open HR → Payroll. Find the run HR prepared in HR-03 and check the totals.
+2. Click Approve. Then Mark paid.</t>
+        </is>
+      </c>
+      <c r="E14" s="38" t="inlineStr">
+        <is>
+          <t>The run is Approved, then Paid, and the wage cost is posted to the books. HR can prepare a run but not approve it, so the salary run is always checked by a second person.</t>
+        </is>
+      </c>
+      <c r="F14" s="40" t="inlineStr">
+        <is>
+          <t>Needs HR-03.</t>
+        </is>
+      </c>
+      <c r="G14" s="41" t="n"/>
+      <c r="H14" s="41" t="n"/>
+      <c r="I14" s="41" t="n"/>
+      <c r="J14" s="41" t="n"/>
+      <c r="K14" s="42" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A7:K13"/>
+  <autoFilter ref="A7:K14"/>
   <mergeCells count="2">
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="C4:D4"/>
   </mergeCells>
-  <conditionalFormatting sqref="G8:G13">
+  <conditionalFormatting sqref="G8:G14">
     <cfRule type="expression" priority="1" dxfId="2">
       <formula>$G8="Pass"</formula>
     </cfRule>
@@ -2291,19 +2326,19 @@
       <formula>$G8="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H8:I13">
+  <conditionalFormatting sqref="H8:I14">
     <cfRule type="expression" priority="4" dxfId="3">
       <formula>AND(OR($G8="Fail",$G8="Blocked"),H8="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="G8:G13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Result" error="Choose Pass, Fail, Blocked or Not run." type="list">
+    <dataValidation sqref="G8:G14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Result" error="Choose Pass, Fail, Blocked or Not run." type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
-    <dataValidation sqref="H8:H13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Severity" error="Choose Critical, Major, Minor or Suggestion." type="list">
+    <dataValidation sqref="H8:H14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Severity" error="Choose Critical, Major, Minor or Suggestion." type="list">
       <formula1>"Critical,Major,Minor,Suggestion"</formula1>
     </dataValidation>
-    <dataValidation sqref="K8:K13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date" error="Enter the date as dd/mm/yyyy." type="date" operator="greaterThan">
+    <dataValidation sqref="K8:K14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date" error="Enter the date as dd/mm/yyyy." type="date" operator="greaterThan">
       <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -2329,7 +2364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2752,13 +2787,48 @@
       <c r="J16" s="41" t="n"/>
       <c r="K16" s="42" t="n"/>
     </row>
+    <row r="17" ht="100.5" customHeight="1">
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t>HR-10</t>
+        </is>
+      </c>
+      <c r="B17" s="38" t="inlineStr">
+        <is>
+          <t>Finance &amp; HR</t>
+        </is>
+      </c>
+      <c r="C17" s="39" t="inlineStr">
+        <is>
+          <t>The HR dashboard: today, and what is waiting</t>
+        </is>
+      </c>
+      <c r="D17" s="38" t="inlineStr">
+        <is>
+          <t>1. Click HR &amp; Admin in the menu. It opens on the Dashboard tab.
+2. Mark today's attendance for two people, then come back to the dashboard.
+3. Raise a leave request for someone and come back again.</t>
+        </is>
+      </c>
+      <c r="E17" s="38" t="inlineStr">
+        <is>
+          <t>Present today goes up by the two you marked, and Not yet marked goes down. Leave to decide counts the new request and lists it with its start date. Documents lapsing lists visas, Emirates IDs, labour cards and passports expiring within 60 days. No salary or pay figure appears anywhere on the dashboard.</t>
+        </is>
+      </c>
+      <c r="F17" s="40" t="inlineStr"/>
+      <c r="G17" s="41" t="n"/>
+      <c r="H17" s="41" t="n"/>
+      <c r="I17" s="41" t="n"/>
+      <c r="J17" s="41" t="n"/>
+      <c r="K17" s="42" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A7:K16"/>
+  <autoFilter ref="A7:K17"/>
   <mergeCells count="2">
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="C4:D4"/>
   </mergeCells>
-  <conditionalFormatting sqref="G8:G16">
+  <conditionalFormatting sqref="G8:G17">
     <cfRule type="expression" priority="1" dxfId="2">
       <formula>$G8="Pass"</formula>
     </cfRule>
@@ -2769,19 +2839,19 @@
       <formula>$G8="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H8:I16">
+  <conditionalFormatting sqref="H8:I17">
     <cfRule type="expression" priority="4" dxfId="3">
       <formula>AND(OR($G8="Fail",$G8="Blocked"),H8="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="G8:G16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Result" error="Choose Pass, Fail, Blocked or Not run." type="list">
+    <dataValidation sqref="G8:G17" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Result" error="Choose Pass, Fail, Blocked or Not run." type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
-    <dataValidation sqref="H8:H16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Severity" error="Choose Critical, Major, Minor or Suggestion." type="list">
+    <dataValidation sqref="H8:H17" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Severity" error="Choose Critical, Major, Minor or Suggestion." type="list">
       <formula1>"Critical,Major,Minor,Suggestion"</formula1>
     </dataValidation>
-    <dataValidation sqref="K8:K16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date" error="Enter the date as dd/mm/yyyy." type="date" operator="greaterThan">
+    <dataValidation sqref="K8:K17" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date" error="Enter the date as dd/mm/yyyy." type="date" operator="greaterThan">
       <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -2960,7 +3030,7 @@
       <c r="J8" s="41" t="n"/>
       <c r="K8" s="42" t="n"/>
     </row>
-    <row r="9" ht="60" customHeight="1">
+    <row r="9" ht="100.5" customHeight="1">
       <c r="A9" s="37" t="inlineStr">
         <is>
           <t>TK-02</t>
@@ -2984,7 +3054,7 @@
       </c>
       <c r="E9" s="38" t="inlineStr">
         <is>
-          <t>The menu shows only the Dashboard and Attendance &amp; Muster. Every other address returns you to the dashboard — no salaries, payroll, employee profiles or finance screens are shown.</t>
+          <t>The menu shows only the Dashboard and HR &amp; Admin. HR &amp; Admin opens an HR dashboard showing only today's muster, with Attendance &amp; Muster as the one other tab. Every other address returns you to the dashboard — no salaries, payroll, employee profiles or finance screens are shown.</t>
         </is>
       </c>
       <c r="F9" s="40" t="inlineStr"/>
@@ -3881,534 +3951,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="32" t="inlineStr">
-        <is>
-          <t>Administrator</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="29" t="inlineStr">
-        <is>
-          <t>Sign in as:</t>
-        </is>
-      </c>
-      <c r="C2" s="30" t="inlineStr">
-        <is>
-          <t>Group Admin</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="33" t="inlineStr">
-        <is>
-          <t>Sets up the companies, the letterhead on printed documents, email, users and who may approve what. Run these first: several other roles depend on them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="29" t="inlineStr">
-        <is>
-          <t>Tester:</t>
-        </is>
-      </c>
-      <c r="C4" s="34" t="n"/>
-      <c r="E4" s="31" t="inlineStr">
-        <is>
-          <t>Yellow cells are yours to fill in. Result and Severity have drop-down lists.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="35" t="inlineStr">
-        <is>
-          <t>← Back to Summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="36" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="B7" s="36" t="inlineStr">
-        <is>
-          <t>Area</t>
-        </is>
-      </c>
-      <c r="C7" s="36" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="D7" s="36" t="inlineStr">
-        <is>
-          <t>Steps</t>
-        </is>
-      </c>
-      <c r="E7" s="36" t="inlineStr">
-        <is>
-          <t>Expected result</t>
-        </is>
-      </c>
-      <c r="F7" s="36" t="inlineStr">
-        <is>
-          <t>Depends on</t>
-        </is>
-      </c>
-      <c r="G7" s="36" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-      <c r="H7" s="36" t="inlineStr">
-        <is>
-          <t>Severity</t>
-        </is>
-      </c>
-      <c r="I7" s="36" t="inlineStr">
-        <is>
-          <t>What actually happened</t>
-        </is>
-      </c>
-      <c r="J7" s="36" t="inlineStr">
-        <is>
-          <t>Tested by</t>
-        </is>
-      </c>
-      <c r="K7" s="36" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="87" customHeight="1">
-      <c r="A8" s="37" t="inlineStr">
-        <is>
-          <t>ADM-01</t>
-        </is>
-      </c>
-      <c r="B8" s="38" t="inlineStr">
-        <is>
-          <t>Finance &amp; HR</t>
-        </is>
-      </c>
-      <c r="C8" s="39" t="inlineStr">
-        <is>
-          <t>Complete a company's legal details</t>
-        </is>
-      </c>
-      <c r="D8" s="38" t="inlineStr">
-        <is>
-          <t>1. Open Companies and edit WBE.
-2. Enter the VAT registration number (TRN) with spaces, as printed on the certificate.
-3. Enter the address line and city, and choose the emirate.
-4. Save, then open the record again.</t>
-        </is>
-      </c>
-      <c r="E8" s="38" t="inlineStr">
-        <is>
-          <t>The details are kept. The TRN is stored without the spaces. The emirate is chosen from the seven, not typed.</t>
-        </is>
-      </c>
-      <c r="F8" s="40" t="inlineStr"/>
-      <c r="G8" s="41" t="n"/>
-      <c r="H8" s="41" t="n"/>
-      <c r="I8" s="41" t="n"/>
-      <c r="J8" s="41" t="n"/>
-      <c r="K8" s="42" t="n"/>
-    </row>
-    <row r="9" ht="127.5" customHeight="1">
-      <c r="A9" s="37" t="inlineStr">
-        <is>
-          <t>ADM-02</t>
-        </is>
-      </c>
-      <c r="B9" s="38" t="inlineStr">
-        <is>
-          <t>CRM, Inventory &amp; documents</t>
-        </is>
-      </c>
-      <c r="C9" s="39" t="inlineStr">
-        <is>
-          <t>Set the letterhead for printed documents</t>
-        </is>
-      </c>
-      <c r="D9" s="38" t="inlineStr">
-        <is>
-          <t>1. Open Settings → Printed Documents and choose WBE at the top.
-2. Set the accent colour, phone, email and website, and a footer line such as the trade licence number.
-3. Paste standard terms into Quotation terms, Purchase order terms and Enquiry (RFQ) terms.
-4. Save.
-5. Click Print next to “See it on paper”.</t>
-        </is>
-      </c>
-      <c r="E9" s="38" t="inlineStr">
-        <is>
-          <t>A PDF opens with SAMPLE across the page, your contact details under the company name, the TRN, the accent colour on the title and rules, your quotation terms, the footer line at the bottom and “Page 1 of 1”.</t>
-        </is>
-      </c>
-      <c r="F9" s="40" t="inlineStr"/>
-      <c r="G9" s="41" t="n"/>
-      <c r="H9" s="41" t="n"/>
-      <c r="I9" s="41" t="n"/>
-      <c r="J9" s="41" t="n"/>
-      <c r="K9" s="42" t="n"/>
-    </row>
-    <row r="10" ht="73.5" customHeight="1">
-      <c r="A10" s="37" t="inlineStr">
-        <is>
-          <t>ADM-03</t>
-        </is>
-      </c>
-      <c r="B10" s="38" t="inlineStr">
-        <is>
-          <t>CRM, Inventory &amp; documents</t>
-        </is>
-      </c>
-      <c r="C10" s="39" t="inlineStr">
-        <is>
-          <t>Use the company's own letterhead artwork</t>
-        </is>
-      </c>
-      <c r="D10" s="38" t="inlineStr">
-        <is>
-          <t>1. On Settings → Printed Documents, choose a PNG or JPEG of the letterhead band as Header artwork.
-2. Save and print the sample again.
-3. Now try choosing an SVG, GIF or PDF file as the artwork.</t>
-        </is>
-      </c>
-      <c r="E10" s="38" t="inlineStr">
-        <is>
-          <t>The sample shows the artwork across the top instead of the name and logo. The SVG, GIF or PDF is refused with a message asking for a PNG or JPEG.</t>
-        </is>
-      </c>
-      <c r="F10" s="40" t="inlineStr"/>
-      <c r="G10" s="41" t="n"/>
-      <c r="H10" s="41" t="n"/>
-      <c r="I10" s="41" t="n"/>
-      <c r="J10" s="41" t="n"/>
-      <c r="K10" s="42" t="n"/>
-    </row>
-    <row r="11" ht="46.5" customHeight="1">
-      <c r="A11" s="37" t="inlineStr">
-        <is>
-          <t>ADM-04</t>
-        </is>
-      </c>
-      <c r="B11" s="38" t="inlineStr">
-        <is>
-          <t>CRM, Inventory &amp; documents</t>
-        </is>
-      </c>
-      <c r="C11" s="39" t="inlineStr">
-        <is>
-          <t>Warnings for missing company details</t>
-        </is>
-      </c>
-      <c r="D11" s="38" t="inlineStr">
-        <is>
-          <t>1. On Settings → Printed Documents, switch to a company with no TRN or no address recorded.</t>
-        </is>
-      </c>
-      <c r="E11" s="38" t="inlineStr">
-        <is>
-          <t>A yellow warning says what is missing and links to Companies. Documents for that company still print, with the name only.</t>
-        </is>
-      </c>
-      <c r="F11" s="40" t="inlineStr"/>
-      <c r="G11" s="41" t="n"/>
-      <c r="H11" s="41" t="n"/>
-      <c r="I11" s="41" t="n"/>
-      <c r="J11" s="41" t="n"/>
-      <c r="K11" s="42" t="n"/>
-    </row>
-    <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="37" t="inlineStr">
-        <is>
-          <t>ADM-05</t>
-        </is>
-      </c>
-      <c r="B12" s="38" t="inlineStr">
-        <is>
-          <t>CRM, Inventory &amp; documents</t>
-        </is>
-      </c>
-      <c r="C12" s="39" t="inlineStr">
-        <is>
-          <t>Connect the mail server</t>
-        </is>
-      </c>
-      <c r="D12" s="38" t="inlineStr">
-        <is>
-          <t>1. Open Settings → Email and choose the provider.
-2. Enter the mailbox, its password or app password, and the send-as name and address.
-3. Save, then Send a test to your own address.</t>
-        </is>
-      </c>
-      <c r="E12" s="38" t="inlineStr">
-        <is>
-          <t>The test email arrives. If it does not, the screen shows the mail server's own message, which can be given to IT. The password is not shown again after saving.</t>
-        </is>
-      </c>
-      <c r="F12" s="40" t="inlineStr">
-        <is>
-          <t>Needs a real mailbox from IT. Mark Blocked if there is none yet.</t>
-        </is>
-      </c>
-      <c r="G12" s="41" t="n"/>
-      <c r="H12" s="41" t="n"/>
-      <c r="I12" s="41" t="n"/>
-      <c r="J12" s="41" t="n"/>
-      <c r="K12" s="42" t="n"/>
-    </row>
-    <row r="13" ht="73.5" customHeight="1">
-      <c r="A13" s="37" t="inlineStr">
-        <is>
-          <t>ADM-06</t>
-        </is>
-      </c>
-      <c r="B13" s="38" t="inlineStr">
-        <is>
-          <t>Finance &amp; HR</t>
-        </is>
-      </c>
-      <c r="C13" s="39" t="inlineStr">
-        <is>
-          <t>Create a login for each tester</t>
-        </is>
-      </c>
-      <c r="D13" s="38" t="inlineStr">
-        <is>
-          <t>1. Open Users and add a user for each role on this page, giving each the role and the companies they work in.
-2. Note the temporary password shown.
-3. Sign in as one of them in a private window.</t>
-        </is>
-      </c>
-      <c r="E13" s="38" t="inlineStr">
-        <is>
-          <t>The temporary password is shown once. The new user must set their own password before they can go any further.</t>
-        </is>
-      </c>
-      <c r="F13" s="40" t="inlineStr"/>
-      <c r="G13" s="41" t="n"/>
-      <c r="H13" s="41" t="n"/>
-      <c r="I13" s="41" t="n"/>
-      <c r="J13" s="41" t="n"/>
-      <c r="K13" s="42" t="n"/>
-    </row>
-    <row r="14" ht="46.5" customHeight="1">
-      <c r="A14" s="37" t="inlineStr">
-        <is>
-          <t>ADM-07</t>
-        </is>
-      </c>
-      <c r="B14" s="38" t="inlineStr">
-        <is>
-          <t>Finance &amp; HR</t>
-        </is>
-      </c>
-      <c r="C14" s="39" t="inlineStr">
-        <is>
-          <t>Access follows the role</t>
-        </is>
-      </c>
-      <c r="D14" s="38" t="inlineStr">
-        <is>
-          <t>1. Sign in as the Storekeeper.
-2. Look at the menu, then type /finance at the end of the address and press Enter.</t>
-        </is>
-      </c>
-      <c r="E14" s="38" t="inlineStr">
-        <is>
-          <t>Finance is not in the menu. Typing the address returns you to the dashboard without showing any of the Finance screen.</t>
-        </is>
-      </c>
-      <c r="F14" s="40" t="inlineStr"/>
-      <c r="G14" s="41" t="n"/>
-      <c r="H14" s="41" t="n"/>
-      <c r="I14" s="41" t="n"/>
-      <c r="J14" s="41" t="n"/>
-      <c r="K14" s="42" t="n"/>
-    </row>
-    <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="37" t="inlineStr">
-        <is>
-          <t>ADM-08</t>
-        </is>
-      </c>
-      <c r="B15" s="38" t="inlineStr">
-        <is>
-          <t>CRM, Inventory &amp; documents</t>
-        </is>
-      </c>
-      <c r="C15" s="39" t="inlineStr">
-        <is>
-          <t>Changing a role's access survives the next release</t>
-        </is>
-      </c>
-      <c r="D15" s="38" t="inlineStr">
-        <is>
-          <t>1. Open Access Control and remove one screen from the Storekeeper role, e.g. Returns from Site.
-2. Ask the project team to note it, and re-check after the next update is deployed to Pre-Prod.</t>
-        </is>
-      </c>
-      <c r="E15" s="38" t="inlineStr">
-        <is>
-          <t>After the update the Storekeeper still does not have that screen. Changes made here are never reset by a new release.</t>
-        </is>
-      </c>
-      <c r="F15" s="40" t="inlineStr">
-        <is>
-          <t>Needs a deployment between the two halves. Leave as Not run until then.</t>
-        </is>
-      </c>
-      <c r="G15" s="41" t="n"/>
-      <c r="H15" s="41" t="n"/>
-      <c r="I15" s="41" t="n"/>
-      <c r="J15" s="41" t="n"/>
-      <c r="K15" s="42" t="n"/>
-    </row>
-    <row r="16" ht="87" customHeight="1">
-      <c r="A16" s="37" t="inlineStr">
-        <is>
-          <t>ADM-09</t>
-        </is>
-      </c>
-      <c r="B16" s="38" t="inlineStr">
-        <is>
-          <t>CRM, Inventory &amp; documents</t>
-        </is>
-      </c>
-      <c r="C16" s="39" t="inlineStr">
-        <is>
-          <t>Approval routes are as agreed</t>
-        </is>
-      </c>
-      <c r="D16" s="38" t="inlineStr">
-        <is>
-          <t>1. Open Approvals → Configure routes.</t>
-        </is>
-      </c>
-      <c r="E16" s="38" t="inlineStr">
-        <is>
-          <t>Material Request: Site Engineer / Planner → Project Manager → Procurement Officer. Purchase Order: Project Manager → Operations Manager → Director, plus Managing Director from AED 50,000. Sales Quotation: Operations Manager → Director, plus Managing Director from AED 500,000.</t>
-        </is>
-      </c>
-      <c r="F16" s="40" t="inlineStr"/>
-      <c r="G16" s="41" t="n"/>
-      <c r="H16" s="41" t="n"/>
-      <c r="I16" s="41" t="n"/>
-      <c r="J16" s="41" t="n"/>
-      <c r="K16" s="42" t="n"/>
-    </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="37" t="inlineStr">
-        <is>
-          <t>ADM-10</t>
-        </is>
-      </c>
-      <c r="B17" s="38" t="inlineStr">
-        <is>
-          <t>Finance &amp; HR</t>
-        </is>
-      </c>
-      <c r="C17" s="39" t="inlineStr">
-        <is>
-          <t>The audit trail shows who changed what</t>
-        </is>
-      </c>
-      <c r="D17" s="38" t="inlineStr">
-        <is>
-          <t>1. Open Audit Log and search for “Printed document settings”.
-2. Search for your own name.</t>
-        </is>
-      </c>
-      <c r="E17" s="38" t="inlineStr">
-        <is>
-          <t>Your change is listed with the time and your name. The artwork itself is not dumped into the log. Nothing in the log can be edited or deleted.</t>
-        </is>
-      </c>
-      <c r="F17" s="40" t="inlineStr"/>
-      <c r="G17" s="41" t="n"/>
-      <c r="H17" s="41" t="n"/>
-      <c r="I17" s="41" t="n"/>
-      <c r="J17" s="41" t="n"/>
-      <c r="K17" s="42" t="n"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A7:K17"/>
-  <mergeCells count="2">
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="C4:D4"/>
-  </mergeCells>
-  <conditionalFormatting sqref="G8:G17">
-    <cfRule type="expression" priority="1" dxfId="2">
-      <formula>$G8="Pass"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="0">
-      <formula>$G8="Fail"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="1">
-      <formula>$G8="Blocked"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H8:I17">
-    <cfRule type="expression" priority="4" dxfId="3">
-      <formula>AND(OR($G8="Fail",$G8="Blocked"),H8="")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="3">
-    <dataValidation sqref="G8:G17" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Result" error="Choose Pass, Fail, Blocked or Not run." type="list">
-      <formula1>"Pass,Fail,Blocked,Not run"</formula1>
-    </dataValidation>
-    <dataValidation sqref="H8:H17" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Severity" error="Choose Critical, Major, Minor or Suggestion." type="list">
-      <formula1>"Critical,Major,Minor,Suggestion"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K8:K17" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date" error="Enter the date as dd/mm/yyyy." type="date" operator="greaterThan">
-      <formula1>DATE(2026,1,1)</formula1>
-    </dataValidation>
-  </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="A5" location="'Summary'!A1" display="← Back to Summary"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;LWB Group ERP Acceptance Scripts · Administrator&amp;RPage &amp;P of &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
   <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4428,7 +3970,7 @@
     <row r="1">
       <c r="A1" s="32" t="inlineStr">
         <is>
-          <t>Estimator / Sales</t>
+          <t>Administrator</t>
         </is>
       </c>
     </row>
@@ -4440,14 +3982,14 @@
       </c>
       <c r="C2" s="30" t="inlineStr">
         <is>
-          <t>Estimation / Sales Engineer</t>
+          <t>Group Admin</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="33" t="inlineStr">
         <is>
-          <t>Takes an enquiry from first call to a priced, approved quotation, and records what the customer ordered.</t>
+          <t>Sets up the companies, the letterhead on printed documents, email, users and who may approve what. Run these first: several other roles depend on them.</t>
         </is>
       </c>
     </row>
@@ -4531,29 +4073,30 @@
     <row r="8" ht="87" customHeight="1">
       <c r="A8" s="37" t="inlineStr">
         <is>
-          <t>EST-01</t>
+          <t>ADM-01</t>
         </is>
       </c>
       <c r="B8" s="38" t="inlineStr">
         <is>
-          <t>CRM, Inventory &amp; documents</t>
+          <t>Finance &amp; HR</t>
         </is>
       </c>
       <c r="C8" s="39" t="inlineStr">
         <is>
-          <t>Log a new enquiry</t>
+          <t>Complete a company's legal details</t>
         </is>
       </c>
       <c r="D8" s="38" t="inlineStr">
         <is>
-          <t>1. Open CRM &amp; Estimation → Pipeline and click Log an enquiry.
-2. Enter a title, choose the customer Deep Port Logistics FZC, the estimated value and where it came from.
-3. Save.</t>
+          <t>1. Open Companies and edit WBE.
+2. Enter the VAT registration number (TRN) with spaces, as printed on the certificate.
+3. Enter the address line and city, and choose the emirate.
+4. Save, then open the record again.</t>
         </is>
       </c>
       <c r="E8" s="38" t="inlineStr">
         <is>
-          <t>The card appears in the first column. The column's weighted total goes up by less than the full value, because a new enquiry is unlikely to be won yet.</t>
+          <t>The details are kept. The TRN is stored without the spaces. The emirate is chosen from the seven, not typed.</t>
         </is>
       </c>
       <c r="F8" s="40" t="inlineStr"/>
@@ -4563,10 +4106,10 @@
       <c r="J8" s="41" t="n"/>
       <c r="K8" s="42" t="n"/>
     </row>
-    <row r="9" ht="60" customHeight="1">
+    <row r="9" ht="127.5" customHeight="1">
       <c r="A9" s="37" t="inlineStr">
         <is>
-          <t>EST-02</t>
+          <t>ADM-02</t>
         </is>
       </c>
       <c r="B9" s="38" t="inlineStr">
@@ -4576,18 +4119,21 @@
       </c>
       <c r="C9" s="39" t="inlineStr">
         <is>
-          <t>Move an enquiry on</t>
+          <t>Set the letterhead for printed documents</t>
         </is>
       </c>
       <c r="D9" s="38" t="inlineStr">
         <is>
-          <t>1. Open your enquiry and click Move it on.
-2. Choose the next stage and read the dialog before confirming.</t>
+          <t>1. Open Settings → Printed Documents and choose WBE at the top.
+2. Set the accent colour, phone, email and website, and a footer line such as the trade licence number.
+3. Paste standard terms into Quotation terms, Purchase order terms and Enquiry (RFQ) terms.
+4. Save.
+5. Click Print next to “See it on paper”.</t>
         </is>
       </c>
       <c r="E9" s="38" t="inlineStr">
         <is>
-          <t>Before you confirm, the dialog shows what the move does to the chance of winning. After it, the card is in the new column and the tracker bar has moved.</t>
+          <t>A PDF opens with SAMPLE across the page, your contact details under the company name, the TRN, the accent colour on the title and rules, your quotation terms, the footer line at the bottom and “Page 1 of 1”.</t>
         </is>
       </c>
       <c r="F9" s="40" t="inlineStr"/>
@@ -4600,7 +4146,7 @@
     <row r="10" ht="73.5" customHeight="1">
       <c r="A10" s="37" t="inlineStr">
         <is>
-          <t>EST-03</t>
+          <t>ADM-03</t>
         </is>
       </c>
       <c r="B10" s="38" t="inlineStr">
@@ -4610,19 +4156,19 @@
       </c>
       <c r="C10" s="39" t="inlineStr">
         <is>
-          <t>Book a site visit, then file the report</t>
+          <t>Use the company's own letterhead artwork</t>
         </is>
       </c>
       <c r="D10" s="38" t="inlineStr">
         <is>
-          <t>1. On the enquiry click Record beside Site visits. Enter the date and who is going; leave findings empty. Save.
-2. Click File the report and save it empty.
-3. File it again with what was found.</t>
+          <t>1. On Settings → Printed Documents, choose a PNG or JPEG of the letterhead band as Header artwork.
+2. Save and print the sample again.
+3. Now try choosing an SVG, GIF or PDF file as the artwork.</t>
         </is>
       </c>
       <c r="E10" s="38" t="inlineStr">
         <is>
-          <t>After booking, the visit shows as booked and the report as still to come. The empty report is refused. With findings, the enquiry shows Site Report Submitted.</t>
+          <t>The sample shows the artwork across the top instead of the name and logo. The SVG, GIF or PDF is refused with a message asking for a PNG or JPEG.</t>
         </is>
       </c>
       <c r="F10" s="40" t="inlineStr"/>
@@ -4632,10 +4178,10 @@
       <c r="J10" s="41" t="n"/>
       <c r="K10" s="42" t="n"/>
     </row>
-    <row r="11" ht="73.5" customHeight="1">
+    <row r="11" ht="46.5" customHeight="1">
       <c r="A11" s="37" t="inlineStr">
         <is>
-          <t>EST-04</t>
+          <t>ADM-04</t>
         </is>
       </c>
       <c r="B11" s="38" t="inlineStr">
@@ -4645,19 +4191,17 @@
       </c>
       <c r="C11" s="39" t="inlineStr">
         <is>
-          <t>Build up an estimate</t>
+          <t>Warnings for missing company details</t>
         </is>
       </c>
       <c r="D11" s="38" t="inlineStr">
         <is>
-          <t>1. Open Estimates and click Start an estimate for your enquiry. Set overhead and margin.
-2. Add a line measured in metres: material cost, labour hours and rate, plant hours and rate.
-3. Add a lump-sum line.</t>
+          <t>1. On Settings → Printed Documents, switch to a company with no TRN or no address recorded.</t>
         </is>
       </c>
       <c r="E11" s="38" t="inlineStr">
         <is>
-          <t>The unit cost adds itself up as you type. The lump-sum line does not ask for a quantity. There is no box to type the selling price.</t>
+          <t>A yellow warning says what is missing and links to Companies. Documents for that company still print, with the name only.</t>
         </is>
       </c>
       <c r="F11" s="40" t="inlineStr"/>
@@ -4667,10 +4211,10 @@
       <c r="J11" s="41" t="n"/>
       <c r="K11" s="42" t="n"/>
     </row>
-    <row r="12" ht="46.5" customHeight="1">
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="37" t="inlineStr">
         <is>
-          <t>EST-05</t>
+          <t>ADM-05</t>
         </is>
       </c>
       <c r="B12" s="38" t="inlineStr">
@@ -4680,52 +4224,58 @@
       </c>
       <c r="C12" s="39" t="inlineStr">
         <is>
-          <t>Take material off with wastage</t>
+          <t>Connect the mail server</t>
         </is>
       </c>
       <c r="D12" s="38" t="inlineStr">
         <is>
-          <t>1. On the metre line click Add material. Enter how much one metre needs and a wastage of 5%.
-2. Save.</t>
+          <t>1. Open Settings → Email and choose the provider.
+2. Enter the mailbox, its password or app password, and the send-as name and address.
+3. Save, then Send a test to your own address.</t>
         </is>
       </c>
       <c r="E12" s="38" t="inlineStr">
         <is>
-          <t>The line's material cost now comes from the takeoff, including the 5% wastage.</t>
-        </is>
-      </c>
-      <c r="F12" s="40" t="inlineStr"/>
+          <t>The test email arrives. If it does not, the screen shows the mail server's own message, which can be given to IT. The password is not shown again after saving.</t>
+        </is>
+      </c>
+      <c r="F12" s="40" t="inlineStr">
+        <is>
+          <t>Needs a real mailbox from IT. Mark Blocked if there is none yet.</t>
+        </is>
+      </c>
       <c r="G12" s="41" t="n"/>
       <c r="H12" s="41" t="n"/>
       <c r="I12" s="41" t="n"/>
       <c r="J12" s="41" t="n"/>
       <c r="K12" s="42" t="n"/>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13" ht="73.5" customHeight="1">
       <c r="A13" s="37" t="inlineStr">
         <is>
-          <t>EST-06</t>
+          <t>ADM-06</t>
         </is>
       </c>
       <c r="B13" s="38" t="inlineStr">
         <is>
-          <t>CRM, Inventory &amp; documents</t>
+          <t>Finance &amp; HR</t>
         </is>
       </c>
       <c r="C13" s="39" t="inlineStr">
         <is>
-          <t>An estimate with nothing costed cannot be priced</t>
+          <t>Create a login for each tester</t>
         </is>
       </c>
       <c r="D13" s="38" t="inlineStr">
         <is>
-          <t>1. Start a second estimate, add a line with no material, labour, plant or subcontract cost.
-2. Click Mark it priced.</t>
+          <t>1. Open Users and add a user for each role on this page, giving each the role and the companies they work in.
+2. Note the temporary password shown.
+3. Sign in as one of them in a private window.</t>
         </is>
       </c>
       <c r="E13" s="38" t="inlineStr">
         <is>
-          <t>Refused: nothing has been costed yet, so there is no price to quote. (A price below cost is also refused unless it is deliberately marked as a loss leader.)</t>
+          <t>The temporary password is shown once. The new user must set their own password before they can go any further.</t>
         </is>
       </c>
       <c r="F13" s="40" t="inlineStr"/>
@@ -4735,31 +4285,31 @@
       <c r="J13" s="41" t="n"/>
       <c r="K13" s="42" t="n"/>
     </row>
-    <row r="14" ht="87" customHeight="1">
+    <row r="14" ht="46.5" customHeight="1">
       <c r="A14" s="37" t="inlineStr">
         <is>
-          <t>EST-07</t>
+          <t>ADM-07</t>
         </is>
       </c>
       <c r="B14" s="38" t="inlineStr">
         <is>
-          <t>CRM, Inventory &amp; documents</t>
+          <t>Finance &amp; HR</t>
         </is>
       </c>
       <c r="C14" s="39" t="inlineStr">
         <is>
-          <t>Raise a quotation and check the draft PDF</t>
+          <t>Access follows the role</t>
         </is>
       </c>
       <c r="D14" s="38" t="inlineStr">
         <is>
-          <t>1. Open Quotations and click Raise a quotation, choosing your priced estimate.
-2. Click Print.</t>
+          <t>1. Sign in as the Storekeeper.
+2. Look at the menu, then type /finance at the end of the address and press Enter.</t>
         </is>
       </c>
       <c r="E14" s="38" t="inlineStr">
         <is>
-          <t>The total comes from the estimate, with no box to change it. The PDF shows DRAFT across every page, the customer, each line with quantity, unit, rate and amount, the total in words and your quotation terms. It shows no cost, margin or markup.</t>
+          <t>Finance is not in the menu. Typing the address returns you to the dashboard without showing any of the Finance screen.</t>
         </is>
       </c>
       <c r="F14" s="40" t="inlineStr"/>
@@ -4769,10 +4319,10 @@
       <c r="J14" s="41" t="n"/>
       <c r="K14" s="42" t="n"/>
     </row>
-    <row r="15" ht="46.5" customHeight="1">
+    <row r="15" ht="60" customHeight="1">
       <c r="A15" s="37" t="inlineStr">
         <is>
-          <t>EST-08</t>
+          <t>ADM-08</t>
         </is>
       </c>
       <c r="B15" s="38" t="inlineStr">
@@ -4782,31 +4332,35 @@
       </c>
       <c r="C15" s="39" t="inlineStr">
         <is>
-          <t>Send a quotation for approval</t>
+          <t>Changing a role's access survives the next release</t>
         </is>
       </c>
       <c r="D15" s="38" t="inlineStr">
         <is>
-          <t>1. Click Send for approval.
-2. Try to issue it before anyone has approved.</t>
+          <t>1. Open Access Control and remove one screen from the Storekeeper role, e.g. Returns from Site.
+2. Ask the project team to note it, and re-check after the next update is deployed to Pre-Prod.</t>
         </is>
       </c>
       <c r="E15" s="38" t="inlineStr">
         <is>
-          <t>The status is Awaiting approval and the PDF still says DRAFT. It cannot be sent to the customer until management has signed it.</t>
-        </is>
-      </c>
-      <c r="F15" s="40" t="inlineStr"/>
+          <t>After the update the Storekeeper still does not have that screen. Changes made here are never reset by a new release.</t>
+        </is>
+      </c>
+      <c r="F15" s="40" t="inlineStr">
+        <is>
+          <t>Needs a deployment between the two halves. Leave as Not run until then.</t>
+        </is>
+      </c>
       <c r="G15" s="41" t="n"/>
       <c r="H15" s="41" t="n"/>
       <c r="I15" s="41" t="n"/>
       <c r="J15" s="41" t="n"/>
       <c r="K15" s="42" t="n"/>
     </row>
-    <row r="16" ht="114" customHeight="1">
+    <row r="16" ht="87" customHeight="1">
       <c r="A16" s="37" t="inlineStr">
         <is>
-          <t>EST-09</t>
+          <t>ADM-09</t>
         </is>
       </c>
       <c r="B16" s="38" t="inlineStr">
@@ -4816,25 +4370,20 @@
       </c>
       <c r="C16" s="39" t="inlineStr">
         <is>
-          <t>Email the approved quotation</t>
+          <t>Approval routes are as agreed</t>
         </is>
       </c>
       <c r="D16" s="38" t="inlineStr">
         <is>
-          <t>1. Once approved, click Email it to the customer.
-2. Tick the customer contact, and send.</t>
+          <t>1. Open Approvals → Configure routes.</t>
         </is>
       </c>
       <c r="E16" s="38" t="inlineStr">
         <is>
-          <t>The status becomes Issued. The customer contact receives an email with the quotation PDF attached. The PDF no longer says DRAFT. The send is listed on Settings → Email.</t>
-        </is>
-      </c>
-      <c r="F16" s="40" t="inlineStr">
-        <is>
-          <t>Needs APR-01 approved, and ADM-05 for real email. Without a mail server the button reads “Issue to the customer” and only records where it went.</t>
-        </is>
-      </c>
+          <t>Material Request: Site Engineer / Planner → Project Manager → Procurement Officer. Purchase Order: Project Manager → Operations Manager → Director, plus Managing Director from AED 50,000. Sales Quotation: Operations Manager → Director, plus Managing Director from AED 500,000.</t>
+        </is>
+      </c>
+      <c r="F16" s="40" t="inlineStr"/>
       <c r="G16" s="41" t="n"/>
       <c r="H16" s="41" t="n"/>
       <c r="I16" s="41" t="n"/>
@@ -4844,28 +4393,28 @@
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="37" t="inlineStr">
         <is>
-          <t>EST-10</t>
+          <t>ADM-10</t>
         </is>
       </c>
       <c r="B17" s="38" t="inlineStr">
         <is>
-          <t>CRM, Inventory &amp; documents</t>
+          <t>Finance &amp; HR</t>
         </is>
       </c>
       <c r="C17" s="39" t="inlineStr">
         <is>
-          <t>Revise an issued quotation</t>
+          <t>The audit trail shows who changed what</t>
         </is>
       </c>
       <c r="D17" s="38" t="inlineStr">
         <is>
-          <t>1. On the issued quotation click Raise a revision.
-2. Print the old one, then the new one.</t>
+          <t>1. Open Audit Log and search for “Printed document settings”.
+2. Search for your own name.</t>
         </is>
       </c>
       <c r="E17" s="38" t="inlineStr">
         <is>
-          <t>The old quotation is marked Superseded and its PDF says SUPERSEDED. The new one is titled Quotation — Revision 2 and goes for approval again.</t>
+          <t>Your change is listed with the time and your name. The artwork itself is not dumped into the log. Nothing in the log can be edited or deleted.</t>
         </is>
       </c>
       <c r="F17" s="40" t="inlineStr"/>
@@ -4875,45 +4424,50 @@
       <c r="J17" s="41" t="n"/>
       <c r="K17" s="42" t="n"/>
     </row>
-    <row r="18" ht="60" customHeight="1">
+    <row r="18" ht="114" customHeight="1">
       <c r="A18" s="37" t="inlineStr">
         <is>
-          <t>EST-11</t>
+          <t>ADM-11</t>
         </is>
       </c>
       <c r="B18" s="38" t="inlineStr">
         <is>
-          <t>CRM, Inventory &amp; documents</t>
+          <t>Finance &amp; HR</t>
         </is>
       </c>
       <c r="C18" s="39" t="inlineStr">
         <is>
-          <t>Record the customer's order</t>
+          <t>Give someone a second company</t>
         </is>
       </c>
       <c r="D18" s="38" t="inlineStr">
         <is>
-          <t>1. On an issued quotation click They ordered it.
-2. Enter their PO number and date, and a value slightly different from the quote.
-3. Confirm.</t>
+          <t>1. Open Users &amp; Roles and click the pencil next to the HR tester.
+2. Tick a second company, e.g. WBTS, and click Save changes.
+3. Sign in as the HR tester and open HR &amp; Admin → People.
+4. Back as administrator, untick every company on the same user and save.</t>
         </is>
       </c>
       <c r="E18" s="38" t="inlineStr">
         <is>
-          <t>The difference is shown while you type and must be confirmed. A job is created at the customer's value, not the quoted one, with a budget taken from the estimate.</t>
-        </is>
-      </c>
-      <c r="F18" s="40" t="inlineStr"/>
+          <t>The user's line shows both companies. The HR tester's Company filter now offers All my companies, WBE and WBTS. With every company unticked the form refuses: “Leave at least one company ticked”. The Audit Log says which company was added.</t>
+        </is>
+      </c>
+      <c r="F18" s="40" t="inlineStr">
+        <is>
+          <t>Put the tester back to WBE only afterwards if other checks expect it.</t>
+        </is>
+      </c>
       <c r="G18" s="41" t="n"/>
       <c r="H18" s="41" t="n"/>
       <c r="I18" s="41" t="n"/>
       <c r="J18" s="41" t="n"/>
       <c r="K18" s="42" t="n"/>
     </row>
-    <row r="19" ht="46.5" customHeight="1">
+    <row r="19" ht="60" customHeight="1">
       <c r="A19" s="37" t="inlineStr">
         <is>
-          <t>EST-12</t>
+          <t>ADM-12</t>
         </is>
       </c>
       <c r="B19" s="38" t="inlineStr">
@@ -4923,18 +4477,18 @@
       </c>
       <c r="C19" s="39" t="inlineStr">
         <is>
-          <t>Record a lost enquiry, and see why work is lost</t>
+          <t>The company is always shown</t>
         </is>
       </c>
       <c r="D19" s="38" t="inlineStr">
         <is>
-          <t>1. Move an enquiry to Lost. Give the reason and who won it.
-2. Open All reports → Where the Work Comes From.</t>
+          <t>1. Sign in as any tester who belongs to one company only.
+2. Open HR &amp; Admin → People, then any dashboard.</t>
         </is>
       </c>
       <c r="E19" s="38" t="inlineStr">
         <is>
-          <t>You cannot mark it lost without a reason. The report groups lost work by reason, ordered by value, and lists who took it.</t>
+          <t>Beside the list is the company name, e.g. “Company: WBE — WB Engineering”. It cannot be changed — there is nothing else to choose — but the screen says whose records these are.</t>
         </is>
       </c>
       <c r="F19" s="40" t="inlineStr"/>
@@ -4974,6 +4528,631 @@
       <formula1>"Critical,Major,Minor,Suggestion"</formula1>
     </dataValidation>
     <dataValidation sqref="K8:K19" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date" error="Enter the date as dd/mm/yyyy." type="date" operator="greaterThan">
+      <formula1>DATE(2026,1,1)</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="A5" location="'Summary'!A1" display="← Back to Summary"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;LWB Group ERP Acceptance Scripts · Administrator&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:K20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="32" t="inlineStr">
+        <is>
+          <t>Estimator / Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>Sign in as:</t>
+        </is>
+      </c>
+      <c r="C2" s="30" t="inlineStr">
+        <is>
+          <t>Estimation / Sales Engineer</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="33" t="inlineStr">
+        <is>
+          <t>Takes an enquiry from first call to a priced, approved quotation, and records what the customer ordered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Tester:</t>
+        </is>
+      </c>
+      <c r="C4" s="34" t="n"/>
+      <c r="E4" s="31" t="inlineStr">
+        <is>
+          <t>Yellow cells are yours to fill in. Result and Severity have drop-down lists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>← Back to Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="36" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B7" s="36" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C7" s="36" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D7" s="36" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E7" s="36" t="inlineStr">
+        <is>
+          <t>Expected result</t>
+        </is>
+      </c>
+      <c r="F7" s="36" t="inlineStr">
+        <is>
+          <t>Depends on</t>
+        </is>
+      </c>
+      <c r="G7" s="36" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="H7" s="36" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="I7" s="36" t="inlineStr">
+        <is>
+          <t>What actually happened</t>
+        </is>
+      </c>
+      <c r="J7" s="36" t="inlineStr">
+        <is>
+          <t>Tested by</t>
+        </is>
+      </c>
+      <c r="K7" s="36" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="87" customHeight="1">
+      <c r="A8" s="37" t="inlineStr">
+        <is>
+          <t>EST-01</t>
+        </is>
+      </c>
+      <c r="B8" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C8" s="39" t="inlineStr">
+        <is>
+          <t>Log a new enquiry</t>
+        </is>
+      </c>
+      <c r="D8" s="38" t="inlineStr">
+        <is>
+          <t>1. Open CRM &amp; Estimation → Pipeline and click Log an enquiry.
+2. Enter a title, choose the customer Deep Port Logistics FZC, the estimated value and where it came from.
+3. Save.</t>
+        </is>
+      </c>
+      <c r="E8" s="38" t="inlineStr">
+        <is>
+          <t>The card appears in the first column. The column's weighted total goes up by less than the full value, because a new enquiry is unlikely to be won yet.</t>
+        </is>
+      </c>
+      <c r="F8" s="40" t="inlineStr"/>
+      <c r="G8" s="41" t="n"/>
+      <c r="H8" s="41" t="n"/>
+      <c r="I8" s="41" t="n"/>
+      <c r="J8" s="41" t="n"/>
+      <c r="K8" s="42" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="37" t="inlineStr">
+        <is>
+          <t>EST-02</t>
+        </is>
+      </c>
+      <c r="B9" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C9" s="39" t="inlineStr">
+        <is>
+          <t>Move an enquiry on</t>
+        </is>
+      </c>
+      <c r="D9" s="38" t="inlineStr">
+        <is>
+          <t>1. Open your enquiry and click Move it on.
+2. Choose the next stage and read the dialog before confirming.</t>
+        </is>
+      </c>
+      <c r="E9" s="38" t="inlineStr">
+        <is>
+          <t>Before you confirm, the dialog shows what the move does to the chance of winning. After it, the card is in the new column and the tracker bar has moved.</t>
+        </is>
+      </c>
+      <c r="F9" s="40" t="inlineStr"/>
+      <c r="G9" s="41" t="n"/>
+      <c r="H9" s="41" t="n"/>
+      <c r="I9" s="41" t="n"/>
+      <c r="J9" s="41" t="n"/>
+      <c r="K9" s="42" t="n"/>
+    </row>
+    <row r="10" ht="73.5" customHeight="1">
+      <c r="A10" s="37" t="inlineStr">
+        <is>
+          <t>EST-03</t>
+        </is>
+      </c>
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C10" s="39" t="inlineStr">
+        <is>
+          <t>Book a site visit, then file the report</t>
+        </is>
+      </c>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>1. On the enquiry click Record beside Site visits. Enter the date and who is going; leave findings empty. Save.
+2. Click File the report and save it empty.
+3. File it again with what was found.</t>
+        </is>
+      </c>
+      <c r="E10" s="38" t="inlineStr">
+        <is>
+          <t>After booking, the visit shows as booked and the report as still to come. The empty report is refused. With findings, the enquiry shows Site Report Submitted.</t>
+        </is>
+      </c>
+      <c r="F10" s="40" t="inlineStr"/>
+      <c r="G10" s="41" t="n"/>
+      <c r="H10" s="41" t="n"/>
+      <c r="I10" s="41" t="n"/>
+      <c r="J10" s="41" t="n"/>
+      <c r="K10" s="42" t="n"/>
+    </row>
+    <row r="11" ht="73.5" customHeight="1">
+      <c r="A11" s="37" t="inlineStr">
+        <is>
+          <t>EST-04</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C11" s="39" t="inlineStr">
+        <is>
+          <t>Build up an estimate</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>1. Open Estimates and click Start an estimate for your enquiry. Set overhead and margin.
+2. Add a line measured in metres: material cost, labour hours and rate, plant hours and rate.
+3. Add a lump-sum line.</t>
+        </is>
+      </c>
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>The unit cost adds itself up as you type. The lump-sum line does not ask for a quantity. There is no box to type the selling price.</t>
+        </is>
+      </c>
+      <c r="F11" s="40" t="inlineStr"/>
+      <c r="G11" s="41" t="n"/>
+      <c r="H11" s="41" t="n"/>
+      <c r="I11" s="41" t="n"/>
+      <c r="J11" s="41" t="n"/>
+      <c r="K11" s="42" t="n"/>
+    </row>
+    <row r="12" ht="46.5" customHeight="1">
+      <c r="A12" s="37" t="inlineStr">
+        <is>
+          <t>EST-05</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C12" s="39" t="inlineStr">
+        <is>
+          <t>Take material off with wastage</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="inlineStr">
+        <is>
+          <t>1. On the metre line click Add material. Enter how much one metre needs and a wastage of 5%.
+2. Save.</t>
+        </is>
+      </c>
+      <c r="E12" s="38" t="inlineStr">
+        <is>
+          <t>The line's material cost now comes from the takeoff, including the 5% wastage.</t>
+        </is>
+      </c>
+      <c r="F12" s="40" t="inlineStr"/>
+      <c r="G12" s="41" t="n"/>
+      <c r="H12" s="41" t="n"/>
+      <c r="I12" s="41" t="n"/>
+      <c r="J12" s="41" t="n"/>
+      <c r="K12" s="42" t="n"/>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t>EST-06</t>
+        </is>
+      </c>
+      <c r="B13" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C13" s="39" t="inlineStr">
+        <is>
+          <t>An estimate with nothing costed cannot be priced</t>
+        </is>
+      </c>
+      <c r="D13" s="38" t="inlineStr">
+        <is>
+          <t>1. Start a second estimate, add a line with no material, labour, plant or subcontract cost.
+2. Click Mark it priced.</t>
+        </is>
+      </c>
+      <c r="E13" s="38" t="inlineStr">
+        <is>
+          <t>Refused: nothing has been costed yet, so there is no price to quote. (A price below cost is also refused unless it is deliberately marked as a loss leader.)</t>
+        </is>
+      </c>
+      <c r="F13" s="40" t="inlineStr"/>
+      <c r="G13" s="41" t="n"/>
+      <c r="H13" s="41" t="n"/>
+      <c r="I13" s="41" t="n"/>
+      <c r="J13" s="41" t="n"/>
+      <c r="K13" s="42" t="n"/>
+    </row>
+    <row r="14" ht="87" customHeight="1">
+      <c r="A14" s="37" t="inlineStr">
+        <is>
+          <t>EST-07</t>
+        </is>
+      </c>
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C14" s="39" t="inlineStr">
+        <is>
+          <t>Raise a quotation and check the draft PDF</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
+        <is>
+          <t>1. Open Quotations and click Raise a quotation, choosing your priced estimate.
+2. Click Print.</t>
+        </is>
+      </c>
+      <c r="E14" s="38" t="inlineStr">
+        <is>
+          <t>The total comes from the estimate, with no box to change it. The PDF shows DRAFT across every page, the customer, each line with quantity, unit, rate and amount, the total in words and your quotation terms. It shows no cost, margin or markup.</t>
+        </is>
+      </c>
+      <c r="F14" s="40" t="inlineStr"/>
+      <c r="G14" s="41" t="n"/>
+      <c r="H14" s="41" t="n"/>
+      <c r="I14" s="41" t="n"/>
+      <c r="J14" s="41" t="n"/>
+      <c r="K14" s="42" t="n"/>
+    </row>
+    <row r="15" ht="46.5" customHeight="1">
+      <c r="A15" s="37" t="inlineStr">
+        <is>
+          <t>EST-08</t>
+        </is>
+      </c>
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C15" s="39" t="inlineStr">
+        <is>
+          <t>Send a quotation for approval</t>
+        </is>
+      </c>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>1. Click Send for approval.
+2. Try to issue it before anyone has approved.</t>
+        </is>
+      </c>
+      <c r="E15" s="38" t="inlineStr">
+        <is>
+          <t>The status is Awaiting approval and the PDF still says DRAFT. It cannot be sent to the customer until management has signed it.</t>
+        </is>
+      </c>
+      <c r="F15" s="40" t="inlineStr"/>
+      <c r="G15" s="41" t="n"/>
+      <c r="H15" s="41" t="n"/>
+      <c r="I15" s="41" t="n"/>
+      <c r="J15" s="41" t="n"/>
+      <c r="K15" s="42" t="n"/>
+    </row>
+    <row r="16" ht="114" customHeight="1">
+      <c r="A16" s="37" t="inlineStr">
+        <is>
+          <t>EST-09</t>
+        </is>
+      </c>
+      <c r="B16" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C16" s="39" t="inlineStr">
+        <is>
+          <t>Email the approved quotation</t>
+        </is>
+      </c>
+      <c r="D16" s="38" t="inlineStr">
+        <is>
+          <t>1. Once approved, click Email it to the customer.
+2. Tick the customer contact, and send.</t>
+        </is>
+      </c>
+      <c r="E16" s="38" t="inlineStr">
+        <is>
+          <t>The status becomes Issued. The customer contact receives an email with the quotation PDF attached. The PDF no longer says DRAFT. The send is listed on Settings → Email.</t>
+        </is>
+      </c>
+      <c r="F16" s="40" t="inlineStr">
+        <is>
+          <t>Needs APR-01 approved, and ADM-05 for real email. Without a mail server the button reads “Issue to the customer” and only records where it went.</t>
+        </is>
+      </c>
+      <c r="G16" s="41" t="n"/>
+      <c r="H16" s="41" t="n"/>
+      <c r="I16" s="41" t="n"/>
+      <c r="J16" s="41" t="n"/>
+      <c r="K16" s="42" t="n"/>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t>EST-10</t>
+        </is>
+      </c>
+      <c r="B17" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C17" s="39" t="inlineStr">
+        <is>
+          <t>Revise an issued quotation</t>
+        </is>
+      </c>
+      <c r="D17" s="38" t="inlineStr">
+        <is>
+          <t>1. On the issued quotation click Raise a revision.
+2. Print the old one, then the new one.</t>
+        </is>
+      </c>
+      <c r="E17" s="38" t="inlineStr">
+        <is>
+          <t>The old quotation is marked Superseded and its PDF says SUPERSEDED. The new one is titled Quotation — Revision 2 and goes for approval again.</t>
+        </is>
+      </c>
+      <c r="F17" s="40" t="inlineStr"/>
+      <c r="G17" s="41" t="n"/>
+      <c r="H17" s="41" t="n"/>
+      <c r="I17" s="41" t="n"/>
+      <c r="J17" s="41" t="n"/>
+      <c r="K17" s="42" t="n"/>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="37" t="inlineStr">
+        <is>
+          <t>EST-11</t>
+        </is>
+      </c>
+      <c r="B18" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C18" s="39" t="inlineStr">
+        <is>
+          <t>Record the customer's order</t>
+        </is>
+      </c>
+      <c r="D18" s="38" t="inlineStr">
+        <is>
+          <t>1. On an issued quotation click They ordered it.
+2. Enter their PO number and date, and a value slightly different from the quote.
+3. Confirm.</t>
+        </is>
+      </c>
+      <c r="E18" s="38" t="inlineStr">
+        <is>
+          <t>The difference is shown while you type and must be confirmed. A job is created at the customer's value, not the quoted one, with a budget taken from the estimate.</t>
+        </is>
+      </c>
+      <c r="F18" s="40" t="inlineStr"/>
+      <c r="G18" s="41" t="n"/>
+      <c r="H18" s="41" t="n"/>
+      <c r="I18" s="41" t="n"/>
+      <c r="J18" s="41" t="n"/>
+      <c r="K18" s="42" t="n"/>
+    </row>
+    <row r="19" ht="46.5" customHeight="1">
+      <c r="A19" s="37" t="inlineStr">
+        <is>
+          <t>EST-12</t>
+        </is>
+      </c>
+      <c r="B19" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C19" s="39" t="inlineStr">
+        <is>
+          <t>Record a lost enquiry, and see why work is lost</t>
+        </is>
+      </c>
+      <c r="D19" s="38" t="inlineStr">
+        <is>
+          <t>1. Move an enquiry to Lost. Give the reason and who won it.
+2. Open All reports → Where the Work Comes From.</t>
+        </is>
+      </c>
+      <c r="E19" s="38" t="inlineStr">
+        <is>
+          <t>You cannot mark it lost without a reason. The report groups lost work by reason, ordered by value, and lists who took it.</t>
+        </is>
+      </c>
+      <c r="F19" s="40" t="inlineStr"/>
+      <c r="G19" s="41" t="n"/>
+      <c r="H19" s="41" t="n"/>
+      <c r="I19" s="41" t="n"/>
+      <c r="J19" s="41" t="n"/>
+      <c r="K19" s="42" t="n"/>
+    </row>
+    <row r="20" ht="87" customHeight="1">
+      <c r="A20" s="37" t="inlineStr">
+        <is>
+          <t>EST-13</t>
+        </is>
+      </c>
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C20" s="39" t="inlineStr">
+        <is>
+          <t>The sales dashboard agrees with the pipeline</t>
+        </is>
+      </c>
+      <c r="D20" s="38" t="inlineStr">
+        <is>
+          <t>1. Click CRM &amp; Estimation in the menu. It opens on the Dashboard tab.
+2. Note Open pipeline and the value beside each stage.
+3. Open the Pipeline tab and add up the open deals in one stage.</t>
+        </is>
+      </c>
+      <c r="E20" s="38" t="inlineStr">
+        <is>
+          <t>The stage value on the dashboard is the sum of that stage's deals on the Pipeline. Likely to win is smaller than Open pipeline. Quotations expiring within 14 days are listed, soonest first, and each line opens the quotation list.</t>
+        </is>
+      </c>
+      <c r="F20" s="40" t="inlineStr"/>
+      <c r="G20" s="41" t="n"/>
+      <c r="H20" s="41" t="n"/>
+      <c r="I20" s="41" t="n"/>
+      <c r="J20" s="41" t="n"/>
+      <c r="K20" s="42" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:K20"/>
+  <mergeCells count="2">
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="C4:D4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G8:G20">
+    <cfRule type="expression" priority="1" dxfId="2">
+      <formula>$G8="Pass"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>$G8="Fail"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>$G8="Blocked"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H8:I20">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>AND(OR($G8="Fail",$G8="Blocked"),H8="")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation sqref="G8:G20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Result" error="Choose Pass, Fail, Blocked or Not run." type="list">
+      <formula1>"Pass,Fail,Blocked,Not run"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H8:H20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Severity" error="Choose Critical, Major, Minor or Suggestion." type="list">
+      <formula1>"Critical,Major,Minor,Suggestion"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K8:K20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date" error="Enter the date as dd/mm/yyyy." type="date" operator="greaterThan">
       <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -5451,7 +5630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -5677,30 +5856,31 @@
       <c r="J10" s="41" t="n"/>
       <c r="K10" s="42" t="n"/>
     </row>
-    <row r="11" ht="46.5" customHeight="1">
+    <row r="11" ht="73.5" customHeight="1">
       <c r="A11" s="37" t="inlineStr">
         <is>
-          <t>SITE-04</t>
+          <t>SITE-05</t>
         </is>
       </c>
       <c r="B11" s="38" t="inlineStr">
         <is>
-          <t>CRM, Inventory &amp; documents</t>
+          <t>Finance &amp; HR</t>
         </is>
       </c>
       <c r="C11" s="39" t="inlineStr">
         <is>
-          <t>A request must ask for something</t>
+          <t>Inventory is in the menu, with only your figures</t>
         </is>
       </c>
       <c r="D11" s="38" t="inlineStr">
         <is>
-          <t>1. Start a new request, remove every line, and click Send for approval.</t>
+          <t>1. Look at the menu for Inventory &amp; SCM and click it.
+2. Look at what the Stores Dashboard shows.</t>
         </is>
       </c>
       <c r="E11" s="38" t="inlineStr">
         <is>
-          <t>It is refused, asking for at least one line saying what is needed and how much.</t>
+          <t>Inventory &amp; SCM is in the menu and opens the Stores Dashboard. It shows stock value, items running low and requests waiting. There is no Purchase orders panel and no supplier prices — those belong to Procurement.</t>
         </is>
       </c>
       <c r="F11" s="40" t="inlineStr"/>
@@ -5710,13 +5890,46 @@
       <c r="J11" s="41" t="n"/>
       <c r="K11" s="42" t="n"/>
     </row>
+    <row r="12" ht="46.5" customHeight="1">
+      <c r="A12" s="37" t="inlineStr">
+        <is>
+          <t>SITE-04</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C12" s="39" t="inlineStr">
+        <is>
+          <t>A request must ask for something</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="inlineStr">
+        <is>
+          <t>1. Start a new request, remove every line, and click Send for approval.</t>
+        </is>
+      </c>
+      <c r="E12" s="38" t="inlineStr">
+        <is>
+          <t>It is refused, asking for at least one line saying what is needed and how much.</t>
+        </is>
+      </c>
+      <c r="F12" s="40" t="inlineStr"/>
+      <c r="G12" s="41" t="n"/>
+      <c r="H12" s="41" t="n"/>
+      <c r="I12" s="41" t="n"/>
+      <c r="J12" s="41" t="n"/>
+      <c r="K12" s="42" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A7:K11"/>
+  <autoFilter ref="A7:K12"/>
   <mergeCells count="2">
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="C4:D4"/>
   </mergeCells>
-  <conditionalFormatting sqref="G8:G11">
+  <conditionalFormatting sqref="G8:G12">
     <cfRule type="expression" priority="1" dxfId="2">
       <formula>$G8="Pass"</formula>
     </cfRule>
@@ -5727,19 +5940,19 @@
       <formula>$G8="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H8:I11">
+  <conditionalFormatting sqref="H8:I12">
     <cfRule type="expression" priority="4" dxfId="3">
       <formula>AND(OR($G8="Fail",$G8="Blocked"),H8="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="G8:G11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Result" error="Choose Pass, Fail, Blocked or Not run." type="list">
+    <dataValidation sqref="G8:G12" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Result" error="Choose Pass, Fail, Blocked or Not run." type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
-    <dataValidation sqref="H8:H11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Severity" error="Choose Critical, Major, Minor or Suggestion." type="list">
+    <dataValidation sqref="H8:H12" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Severity" error="Choose Critical, Major, Minor or Suggestion." type="list">
       <formula1>"Critical,Major,Minor,Suggestion"</formula1>
     </dataValidation>
-    <dataValidation sqref="K8:K11" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date" error="Enter the date as dd/mm/yyyy." type="date" operator="greaterThan">
+    <dataValidation sqref="K8:K12" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date" error="Enter the date as dd/mm/yyyy." type="date" operator="greaterThan">
       <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -6561,7 +6774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7057,13 +7270,47 @@
       <c r="J18" s="41" t="n"/>
       <c r="K18" s="42" t="n"/>
     </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="37" t="inlineStr">
+        <is>
+          <t>STR-12</t>
+        </is>
+      </c>
+      <c r="B19" s="38" t="inlineStr">
+        <is>
+          <t>CRM, Inventory &amp; documents</t>
+        </is>
+      </c>
+      <c r="C19" s="39" t="inlineStr">
+        <is>
+          <t>The stores dashboard shows what is running low</t>
+        </is>
+      </c>
+      <c r="D19" s="38" t="inlineStr">
+        <is>
+          <t>1. Open an item and set its reorder level above what is on hand. Save.
+2. Click Inventory &amp; SCM in the menu to open the Stores Dashboard.</t>
+        </is>
+      </c>
+      <c r="E19" s="38" t="inlineStr">
+        <is>
+          <t>Running low counts that item, and it is listed with what is on hand against its reorder level, the lowest first. Stock value by store adds up to the total on the Stock on Hand screen.</t>
+        </is>
+      </c>
+      <c r="F19" s="40" t="inlineStr"/>
+      <c r="G19" s="41" t="n"/>
+      <c r="H19" s="41" t="n"/>
+      <c r="I19" s="41" t="n"/>
+      <c r="J19" s="41" t="n"/>
+      <c r="K19" s="42" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A7:K18"/>
+  <autoFilter ref="A7:K19"/>
   <mergeCells count="2">
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="C4:D4"/>
   </mergeCells>
-  <conditionalFormatting sqref="G8:G18">
+  <conditionalFormatting sqref="G8:G19">
     <cfRule type="expression" priority="1" dxfId="2">
       <formula>$G8="Pass"</formula>
     </cfRule>
@@ -7074,19 +7321,19 @@
       <formula>$G8="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H8:I18">
+  <conditionalFormatting sqref="H8:I19">
     <cfRule type="expression" priority="4" dxfId="3">
       <formula>AND(OR($G8="Fail",$G8="Blocked"),H8="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="G8:G18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Result" error="Choose Pass, Fail, Blocked or Not run." type="list">
+    <dataValidation sqref="G8:G19" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Result" error="Choose Pass, Fail, Blocked or Not run." type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
     </dataValidation>
-    <dataValidation sqref="H8:H18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Severity" error="Choose Critical, Major, Minor or Suggestion." type="list">
+    <dataValidation sqref="H8:H19" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Severity" error="Choose Critical, Major, Minor or Suggestion." type="list">
       <formula1>"Critical,Major,Minor,Suggestion"</formula1>
     </dataValidation>
-    <dataValidation sqref="K8:K18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date" error="Enter the date as dd/mm/yyyy." type="date" operator="greaterThan">
+    <dataValidation sqref="K8:K19" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date" error="Enter the date as dd/mm/yyyy." type="date" operator="greaterThan">
       <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>